<commit_message>
feat: tick hunger and thirst in update_needs, with UT-003 and UT-039 to UT-041
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4591" uniqueCount="2394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4614" uniqueCount="2405">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">38 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">41 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -7531,6 +7531,39 @@
   </si>
   <si>
     <t xml:space="preserve">Needs is an EnumMap&lt;Need, f32&gt; from enum-map, so ALG-02 clamps every value through values_mut instead of a clamp_all of its own.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thirst 0, thirst_per_h 10, 2 game hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thirst 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">appetite 50, hunger_per_h 10, 1 game hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunger 10 (factor 1.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunger 95, rates 10, 10 game hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunger and thirst 100, never more</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-003 is written; new UT-039…041 for update_needs (API-COR-002): thirst rises by the rate per game hour, average appetite keeps the species hunger rate, a need never passes 100; 41 unit test cases.</t>
   </si>
 </sst>
 </file>
@@ -8063,7 +8096,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2392</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12353,7 +12386,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12563,6 +12596,20 @@
       </c>
       <c r="D16" s="4" t="s">
         <v>2393</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>2403</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>2404</v>
       </c>
     </row>
   </sheetData>
@@ -13923,7 +13970,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -14767,6 +14814,69 @@
         <v>2388</v>
       </c>
       <c r="G42" s="4"/>
+    </row>
+    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>2394</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>2395</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>2396</v>
+      </c>
+      <c r="G43" s="4"/>
+    </row>
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>2397</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>2398</v>
+      </c>
+      <c r="G44" s="4"/>
+    </row>
+    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>2400</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>2401</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>2402</v>
+      </c>
+      <c r="G45" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: add WorldView and tick heat and the urge to sing by the hour
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4614" uniqueCount="2405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4641" uniqueCount="2419">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">41 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">45 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -7564,6 +7564,48 @@
   </si>
   <si>
     <t xml:space="preserve">UT-003 is written; new UT-039…041 for update_needs (API-COR-002): thirst rises by the rate per game hour, average appetite keeps the species hunger rate, a need never passes 100; 41 unit test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heat 0, middle of the hot hours (13.5 h), 1 game hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heat 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heat 15, 2 h at night, 1 game hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heat 0, never below</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">urge to sing 0, middle of the morning (7.5 h) and of the evening (17.5 h) song hours, 0.5 game hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">urge to sing 45 at both</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">urge to sing 100, noon, 1 game hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">urge to sing 50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New UT-042…045 for update_needs (API-COR-002): heat rises in the hot hours and stops at 0 at night, the urge to sing rises at dawn and dusk and drops at midday; 45 unit test cases.</t>
   </si>
 </sst>
 </file>
@@ -8096,7 +8138,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2403</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12386,7 +12428,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12610,6 +12652,20 @@
       </c>
       <c r="D17" s="4" t="s">
         <v>2404</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>2417</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>2418</v>
       </c>
     </row>
   </sheetData>
@@ -13970,7 +14026,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -14877,6 +14933,90 @@
         <v>2402</v>
       </c>
       <c r="G45" s="4"/>
+    </row>
+    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
+        <v>2405</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>2406</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>2407</v>
+      </c>
+      <c r="G46" s="4"/>
+    </row>
+    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>2408</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>2409</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>2410</v>
+      </c>
+      <c r="G47" s="4"/>
+    </row>
+    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>2411</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>2412</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>2413</v>
+      </c>
+      <c r="G48" s="4"/>
+    </row>
+    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>2414</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>2415</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>2416</v>
+      </c>
+      <c r="G49" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: tick fatigue by the species routine, with active_windows and is_active_hour
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4641" uniqueCount="2419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4662" uniqueCount="2430">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">45 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">48 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -7606,6 +7606,39 @@
   </si>
   <si>
     <t xml:space="preserve">New UT-042…045 for update_needs (API-COR-002): heat rises in the hot hours and stops at 0 at night, the urge to sing rises at dawn and dusk and drops at midday; 45 unit test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nocturnal (20–6) checked at 23 h, 3 h and 12 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">active, active, not active</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fatigue 0, energy 45, Diurnal, noon, 1 game hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fatigue rises at the species rate (factor 1.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same animal at 2 h, outside the active hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fatigue rises 1.6 × the species rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New UT-046 for active_windows (a window past midnight) and UT-047…048 for update_needs (fatigue at the species rate in the active hours, 1.6 × outside them); 48 unit test cases.</t>
   </si>
 </sst>
 </file>
@@ -8138,7 +8171,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2417</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12428,7 +12461,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12666,6 +12699,20 @@
       </c>
       <c r="D18" s="4" t="s">
         <v>2418</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>2428</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>2429</v>
       </c>
     </row>
   </sheetData>
@@ -14026,7 +14073,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15017,6 +15064,69 @@
         <v>2416</v>
       </c>
       <c r="G49" s="4"/>
+    </row>
+    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>2419</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>730</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>731</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>2420</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>2421</v>
+      </c>
+      <c r="G50" s="4"/>
+    </row>
+    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="s">
+        <v>2422</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>2423</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>2424</v>
+      </c>
+      <c r="G51" s="4"/>
+    </row>
+    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
+        <v>2425</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>2426</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>2427</v>
+      </c>
+      <c r="G52" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: add routine_factor, with UT-049
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4662" uniqueCount="2430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4671" uniqueCount="2435">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">48 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">49 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -7639,6 +7639,21 @@
   </si>
   <si>
     <t xml:space="preserve">New UT-046 for active_windows (a window past midnight) and UT-047…048 for update_needs (fatigue at the species rate in the active hours, 1.6 × outside them); 48 unit test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diurnal: rest and non-rest at noon, rest and non-rest at 2 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.0, 1.0, 1.6, 0.35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New UT-049 for routine_factor (API-COR-018): each branch of the daily rhythm; 49 unit test cases.</t>
   </si>
 </sst>
 </file>
@@ -8171,7 +8186,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2428</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12461,7 +12476,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12713,6 +12728,20 @@
       </c>
       <c r="D19" s="4" t="s">
         <v>2429</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>2433</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>2434</v>
       </c>
     </row>
   </sheetData>
@@ -14073,7 +14102,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15127,6 +15156,27 @@
         <v>2427</v>
       </c>
       <c r="G52" s="4"/>
+    </row>
+    <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="s">
+        <v>2430</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>726</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>727</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>2431</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>2432</v>
+      </c>
+      <c r="G53" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: add the driving values of ALG-10, with fear on the agent and UT-050 to UT-054
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4671" uniqueCount="2435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4704" uniqueCount="2453">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">49 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">54 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -7654,6 +7654,60 @@
   </si>
   <si>
     <t xml:space="preserve">New UT-049 for routine_factor (API-COR-018): each branch of the daily rhythm; 49 unit test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunger 70; safety 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunger pulls 70; safety pulls 70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fatigue 40, Diurnal: noon; 2 h; 2 h limping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40; 95; 130</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fear felt 50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fear pulls 65; calm pulls 27.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">curiosity and energy traits 50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">curiosity pulls 50; boredom pulls 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mark and fight needs 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">both pull 0 (no scent marks or fights yet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">choose_activity (drive)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New UT-050…054 for the driving values of ALG-10 (drive, inside API-COR-009 choose_activity): a need pulls by its value, safety by its lack, fatigue more off hours and when limping, fear and calm by the fear felt now, curiosity and boredom by the traits, mark and fight not yet; 54 unit test cases.</t>
   </si>
 </sst>
 </file>
@@ -8186,7 +8240,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2433</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12476,7 +12530,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12742,6 +12796,20 @@
       </c>
       <c r="D20" s="4" t="s">
         <v>2434</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>2451</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>2452</v>
       </c>
     </row>
   </sheetData>
@@ -14102,7 +14170,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15177,6 +15245,111 @@
         <v>2432</v>
       </c>
       <c r="G53" s="4"/>
+    </row>
+    <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
+        <v>2435</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>2450</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>2436</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>2437</v>
+      </c>
+      <c r="G54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
+        <v>2438</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>2450</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>2439</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>2440</v>
+      </c>
+      <c r="G55" s="4"/>
+    </row>
+    <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>2441</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>2450</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>2442</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>2443</v>
+      </c>
+      <c r="G56" s="4"/>
+    </row>
+    <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4" t="s">
+        <v>2444</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>2450</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>2445</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>2446</v>
+      </c>
+      <c r="G57" s="4"/>
+    </row>
+    <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="4" t="s">
+        <v>2447</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>2450</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>2448</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>2449</v>
+      </c>
+      <c r="G58" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: choose the next activity by Utility score, with UT-055 to UT-058
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4704" uniqueCount="2453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4731" uniqueCount="2467">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">54 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">58 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -6089,10 +6089,10 @@
 Called by apply_effect for each agent in the alarm radius.</t>
   </si>
   <si>
-    <t xml:space="preserve">fn choose_activity(a: &amp;mut Agent, sp: &amp;Species, hour: f32, out: &amp;mut Outbox) -&gt; (ActivityId, Scores)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALG-10 with a.rng; think_agent passes hour = view.hour(); options are looked up in sp.activities; runs only while the state is Choosing.
+    <t xml:space="preserve">fn choose_activity(a: &amp;mut Agent, sp: &amp;Species, hour: f32, out: &amp;mut Outbox) -&gt; Option&lt;(ActivityId, Scores)&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALG-10 with a.rng; think_agent passes hour = view.hour(); options are looked up in sp.activities; runs only while the state is Choosing; None when no option is in sp.activities.
 Chose goes to out.events.</t>
   </si>
   <si>
@@ -7708,6 +7708,48 @@
   </si>
   <si>
     <t xml:space="preserve">New UT-050…054 for the driving values of ALG-10 (drive, inside API-COR-009 choose_activity): a need pulls by its value, safety by its lack, fatigue more off hours and when limping, fear and calm by the fear felt now, curiosity and boredom by the traits, mark and fight not yet; 54 unit test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunger 80, thirst 20; options eat and drink, linear, no noise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eat, with both scores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">two activities with the same score, options in reverse order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the name first in alphabetical order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no options; an option missing from sp.activities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None, no panic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same agent and seed twice, noise 0.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same choice and scores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-COR-009 choose_activity returns Option&lt;(ActivityId, Scores)&gt;: None when no option is in sp.activities, instead of an empty name; new UT-055…058 (highest wins, tie to the first name, nothing to choose, same seed same scores); 58 unit test cases.</t>
   </si>
 </sst>
 </file>
@@ -8240,7 +8282,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2451</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12530,7 +12572,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12810,6 +12852,20 @@
       </c>
       <c r="D21" s="4" t="s">
         <v>2452</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>2465</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>2466</v>
       </c>
     </row>
   </sheetData>
@@ -14170,7 +14226,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15350,6 +15406,90 @@
         <v>2449</v>
       </c>
       <c r="G58" s="4"/>
+    </row>
+    <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4" t="s">
+        <v>2453</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>687</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>2454</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>2455</v>
+      </c>
+      <c r="G59" s="4"/>
+    </row>
+    <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="s">
+        <v>2456</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>687</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>2457</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>2458</v>
+      </c>
+      <c r="G60" s="4"/>
+    </row>
+    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4" t="s">
+        <v>2459</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>687</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>2283</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>2460</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>2461</v>
+      </c>
+      <c r="G61" s="4"/>
+    </row>
+    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4" t="s">
+        <v>2462</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>687</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>2463</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>2464</v>
+      </c>
+      <c r="G62" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: run a step and lower its need, with UT-059 to UT-061; tidy the section order
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4731" uniqueCount="2467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4752" uniqueCount="2478">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">58 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">61 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -6119,7 +6119,7 @@
   <si>
     <t xml:space="preserve">1. On start: duration = a.rng.range(min,max); SimEvent::Anim to out.events.
 2. Move steps: target from memory or perception; fail if none or on MoveFailed → choose again.
-3. Act steps: lower need while running.
+3. Act steps lower their need while running, per second: Eat hunger 14, Drink thirst 20, Rest fatigue 9, Wallow heat 14, Sing urge to sing 20 (from the prototype); other steps lower none. Checks come first, so a step that fails changes nothing.
 4. Done when time over or target reached.</t>
   </si>
   <si>
@@ -7750,6 +7750,39 @@
   </si>
   <si>
     <t xml:space="preserve">API-COR-009 choose_activity returns Option&lt;(ActivityId, Scores)&gt;: None when no option is in sp.activities, instead of an empty name; new UT-055…058 (highest wins, tie to the first name, nothing to choose, same seed same scores); 58 unit test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunger 50, Eat step of 3 s, run 1 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunger 36 (−14 per s), Running</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-060</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same step run twice for 2 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running, then Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a GoTo step; an Eat step while the animal is choosing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed, the animal unchanged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-COR-011 run_step: the steps that lower a need and how fast (Eat, Drink, Rest, Wallow, Sing, from the prototype); it checks before it changes, so a failure leaves the animal unchanged; new UT-059…061; 61 unit test cases.</t>
   </si>
 </sst>
 </file>
@@ -8282,7 +8315,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2465</v>
+        <v>2476</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12572,7 +12605,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12866,6 +12899,20 @@
       </c>
       <c r="D22" s="4" t="s">
         <v>2466</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>2477</v>
       </c>
     </row>
   </sheetData>
@@ -14226,7 +14273,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15490,6 +15537,69 @@
         <v>2464</v>
       </c>
       <c r="G62" s="4"/>
+    </row>
+    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="s">
+        <v>2467</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>2468</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>2469</v>
+      </c>
+      <c r="G63" s="4"/>
+    </row>
+    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
+        <v>2470</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>2471</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>2472</v>
+      </c>
+      <c r="G64" s="4"/>
+    </row>
+    <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
+        <v>2473</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>2283</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>2474</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>2475</v>
+      </c>
+      <c r="G65" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: enter and run an activity step by step, with UT-062 to UT-064
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4752" uniqueCount="2478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4773" uniqueCount="2490">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">61 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">64 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -6117,7 +6117,7 @@
     <t xml:space="preserve">Running|Done|Failed</t>
   </si>
   <si>
-    <t xml:space="preserve">1. On start: duration = a.rng.range(min,max); SimEvent::Anim to out.events.
+    <t xml:space="preserve">1. On entering a step (enter_step): duration = a.rng.range(min, max); SimEvent::Anim to out.events; past the last step the activity ends and the agent is Choosing. do_activity runs the current step: Done enters the next, Failed goes back to Choosing.
 2. Move steps: target from memory or perception; fail if none or on MoveFailed → choose again.
 3. Act steps lower their need while running, per second: Eat hunger 14, Drink thirst 20, Rest fatigue 9, Wallow heat 14, Sing urge to sing 20 (from the prototype); other steps lower none. Checks come first, so a step that fails changes nothing.
 4. Done when time over or target reached.</t>
@@ -7783,6 +7783,42 @@
   </si>
   <si>
     <t xml:space="preserve">API-COR-011 run_step: the steps that lower a need and how fast (Eat, Drink, Rest, Wallow, Sing, from the prototype); it checks before it changes, so a failure leaves the animal unchanged; new UT-059…061; 61 unit test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enter step 0 of a two-step activity; enter step 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">in step 0 with its time within secs; choosing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a two-step activity run with dt longer than each step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">step 0, then step 1, then choosing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-064</t>
+  </si>
+  <si>
+    <t xml:space="preserve">an activity whose first step is GoTo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">back to choosing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-COR-011: the step's time is drawn when the animal enters it (enter_step), and do_activity runs the current step for PRC-11, moving to the next on Done and back to choosing on Failed; new UT-062…064; 64 unit test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">run_step (enter_step, do_activity)</t>
   </si>
 </sst>
 </file>
@@ -8315,7 +8351,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2476</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12605,7 +12641,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12913,6 +12949,20 @@
       </c>
       <c r="D23" s="4" t="s">
         <v>2477</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>2487</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>2488</v>
       </c>
     </row>
   </sheetData>
@@ -14273,7 +14323,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15600,6 +15650,69 @@
         <v>2475</v>
       </c>
       <c r="G65" s="4"/>
+    </row>
+    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="s">
+        <v>2478</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>2489</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>2479</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>2480</v>
+      </c>
+      <c r="G66" s="4"/>
+    </row>
+    <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="4" t="s">
+        <v>2481</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>2489</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>2482</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>2483</v>
+      </c>
+      <c r="G67" s="4"/>
+    </row>
+    <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="s">
+        <v>2484</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>2489</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>2283</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>2485</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>2486</v>
+      </c>
+      <c r="G68" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: keep fatigue from rising while resting, with UT-065
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4773" uniqueCount="2490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4782" uniqueCount="2495">
   <si>
     <t xml:space="preserve">Noetic — Detailed Design</t>
   </si>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">8 Unit Tests</t>
   </si>
   <si>
-    <t xml:space="preserve">64 unit test cases (normal, boundary, abnormal)</t>
+    <t xml:space="preserve">65 unit test cases (normal, boundary, abnormal)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Conventions</t>
@@ -7819,6 +7819,21 @@
   </si>
   <si>
     <t xml:space="preserve">run_step (enter_step, do_activity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UT-065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fatigue 0, in a Rest step at 2 h, 1 game hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fatigue still 0 (no rise while resting)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALG-02 `resting` is the animal in an activity whose current step is Rest (is_resting); new UT-065 for update_needs; 65 unit test cases.</t>
   </si>
 </sst>
 </file>
@@ -8351,7 +8366,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>2487</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12641,7 +12656,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12963,6 +12978,20 @@
       </c>
       <c r="D24" s="4" t="s">
         <v>2488</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>2493</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>2494</v>
       </c>
     </row>
   </sheetData>
@@ -14323,7 +14352,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15713,6 +15742,27 @@
         <v>2486</v>
       </c>
       <c r="G68" s="4"/>
+    </row>
+    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
+        <v>2490</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>2491</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>2492</v>
+      </c>
+      <c r="G69" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
feat: add tick, which moves the clock and has every agent think and act, with UT-066 to UT-068
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -8365,16 +8365,20 @@
       <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>2493</v>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.23</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>2390</v>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-20</t>
+        </is>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12656,7 +12660,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -12992,6 +12996,28 @@
       </c>
       <c r="D25" s="4" t="s">
         <v>2494</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.23</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-20</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-COR-001 tick: the clock moves on and wraps at 24 h, then every animal thinks and acts in id order; an animal whose species is missing stays idle (NFR-12). Until think_due, SimEvent and Effect exist, every animal thinks on every step and tick returns nothing; new UT-066…068; 68 unit test cases.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -14352,7 +14378,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15763,6 +15789,105 @@
         <v>2492</v>
       </c>
       <c r="G69" s="4"/>
+    </row>
+    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-066</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-COR-001</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tick</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clock at 23.5 h, one game hour</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clock at 0.5 h (wraps past midnight)</t>
+        </is>
+      </c>
+      <c r="G70" s="4"/>
+    </row>
+    <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-067</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-COR-001</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tick</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">an animal of a species not in the world, beside one of a known species</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">that animal unchanged, no panic; the other thirstier</t>
+        </is>
+      </c>
+      <c r="G71" s="4"/>
+    </row>
+    <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-068</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-COR-001</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tick</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">secs_per_game_hour 0, one step</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clock and needs unchanged</t>
+        </is>
+      </c>
+      <c r="G72" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -16012,8 +16137,10 @@
       <c r="B22" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>82</v>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">68 unit test cases (normal, boundary, abnormal)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: keep a step from lowering a need below 0, with UT-069
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -8367,7 +8367,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.23</t>
+          <t xml:space="preserve">0.24</t>
         </is>
       </c>
     </row>
@@ -12660,7 +12660,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -13017,6 +13017,28 @@
       <c r="D26" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">API-COR-001 tick: the clock moves on and wraps at 24 h, then every animal thinks and acts in id order; an animal whose species is missing stays idle (NFR-12). Until think_due, SimEvent and Effect exist, every animal thinks on every step and tick returns nothing; new UT-066…068; 68 unit test cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.24</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-20</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-COR-011 run_step lowers a need down to 0 and never below it; it went negative while the animal rested until the next update_needs clamped it. New UT-069; 69 unit test cases.</t>
         </is>
       </c>
     </row>
@@ -14378,7 +14400,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -15888,6 +15910,39 @@
         </is>
       </c>
       <c r="G72" s="4"/>
+    </row>
+    <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-069</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API-COR-011</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">run_step</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hunger 50, Eat step run long enough to take off 100</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hunger 0, never below</t>
+        </is>
+      </c>
+      <c r="G73" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -16139,7 +16194,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">68 unit test cases (normal, boundary, abnormal)</t>
+          <t xml:space="preserve">69 unit test cases (normal, boundary, abnormal)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: pin the golden state of the default world, with UT-025
</commit_message>
<xml_diff>
--- a/docs/05_detailed_design.xlsx
+++ b/docs/05_detailed_design.xlsx
@@ -8367,7 +8367,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.24</t>
+          <t xml:space="preserve">0.25</t>
         </is>
       </c>
     </row>
@@ -12660,7 +12660,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -13039,6 +13039,28 @@
       <c r="D27" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">API-COR-011 run_step lowers a need down to 0 and never below it; it went negative while the animal rested until the next update_needs clamped it. New UT-069; 69 unit test cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.25</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-20</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-025 is written (noetic_core/tests/golden.rs): the default world is four diurnal rabbits that graze, drink and rest, seeds 42…45, from 6 h, 1000 ticks of 0.5 s; the state hash is FNV-1a 64 over the world printed with Debug, since DefaultHasher may change between Rust releases. M1 done.</t>
         </is>
       </c>
     </row>

</xml_diff>